<commit_message>
chore: update news radar report 2026-10-08
</commit_message>
<xml_diff>
--- a/docs/data/rxbenefits_intel_hub_report_2026-10-08.xlsx
+++ b/docs/data/rxbenefits_intel_hub_report_2026-10-08.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -477,357 +477,27 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>340B Rebate Pilot Launches New Compliance Era for Drug Manufacturers</t>
+          <t>Eli Lilly Expands Legal Crackdown on Unauthorized Compounded Weight-Loss Drugs</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>A new 340B rebate pilot program is officially underway, introducing complex tracking and operational requirements for stakeholders navigating the 340B drug pricing landscape. This development impacts pharmaceutical distribution mechanics and compliance strategies that indirectly influence overall commercial pharmacy benefit costs and supply chain dynamics.</t>
+          <t>Eli Lilly has filed additional lawsuits against medical spas and compounding pharmacies selling unapproved versions of its GLP-1 medications like tirzepatide. For self-funded employers and PBMs managing surging obesity drug costs, this crackdown impacts employee access to lower-cost alternatives amid ongoing supply and coverage pressures.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>JDSupra</t>
+          <t>Bloomberg Law News</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Wed, 07 Oct 2026 15:37:05 GMT</t>
+          <t>Thu, 08 Oct 2026 14:14:00 GMT</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxPRXRPVmNYbU9zWElmaERGck1VOHh4MHp2Y2diMU52YjJBcy0xTUxxV3gyendyLVphUTNrbnd5R3pCdnkzbUltclFYWmRMaXdmLW5MQlVIekhxUGJSM0VQY3RuMjB5WkpWN2RSM0JlcHJGVUJURGJ4SmUtLXhwVThwZFZfNEswZ0xH?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>New 340B Rebate Pilot Launches Amid Ongoing Industry Scrutiny</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>A new 340B rebate pilot has officially launched, initiating compliance deadlines and operational shifts for stakeholders managing drug pricing programs. This development directly impacts the 340B program landscape, which heavily influences drug cost dynamics and savings opportunities for self-funded employer health plans. Plan sponsors must monitor how these manufacturer rebate models affect contract pharmacy arrangements and overall specialty drug spend.</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>The National Law Review</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Wed, 07 Oct 2026 17:12:31 GMT</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE9wRjFQTjc2aUFxeWZQZU1feUduaEZUekdETmEwQ3Nlcjh0TTVWVG1mV253NlFQempMUGFFRWZYX055RHZRRF9ZNFN4UFlzdmNvbnFrcDM5YUJ0VEJBZk14WTZFVXdQUVZGYzA5V283VGZTTkYwRDRjc3V2RdIBe0FVX3lxTE9wRjFQTjc2aUFxeWZQZU1feUduaEZUekdETmEwQ3Nlcjh0TTVWVG1mV253NlFQempMUGFFRWZYX055RHZRRF9ZNFN4UFlzdmNvbnFrcDM5YUJ0VEJBZk14WTZFVXdQUVZGYzA5V283VGZTTkYwRDRjc3V2RQ?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Gross-to-Net Realities Reveal Evolving Dynamics for Top Drugmakers</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>An analysis of recent gross-to-net pricing data from leading drug manufacturers highlights ongoing trends in rebates, discounts, and the broader net-pricing channel. This shift directly impacts how self-funded employers and PBMs evaluate net drug spend versus list prices in plan design. The insights are crucial for pharmacy benefit managers navigating cost containment strategies for self-funded plans.</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Drug Channels</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Wed, 07 Oct 2026 09:30:00 GMT</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxQY05yRHRQaWYtZ0hKc29heDEtb05aMEcwQXp0bzJ1Q3A4RkdDOFlLcGJQM0NGV1Z6ZkFDejJuVWFMbE13SDZubUxhcC1SbUVPV0hOSENVRDhJMThRTHNTbFg4cU8xRjB5RWptcmh3NE9SX3dMTnVocEJobm9vNXY1Z0VCZ0E?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Rising PBM Rebates Fail to Curb Climbing Employer Drug Costs</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>As pharmacy benefit manager rebates continue to increase, self-funded employers report that overall drug costs keep climbing, intensifying pressure on plan sponsors to seek greater transparency. This dynamic highlights ongoing friction in net versus gross drug spend management for commercial health plans.</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Human Resources Director</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Wed, 07 Oct 2026 01:40:14 GMT</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQY0F0MnVvNWdqVEFyODRWU2c5SXpkUlREM21oQ0oyYkhrZWNmSzRIWXF0LTI5aHF5UGhlV0lLekpfV0c2S3lGNjhwWElyNGYtajZ1Y3JkS2Y0R2R4dkREdDdYcDl5cVJuTFRKZ0RRUDB5X3RPQWJsR29vbkh4aURWYW5HVE1GdlE5aDRZNm8tTnpqTVEtZmU3T2FFa3hwcWhtQXdpVTZ1bEVxWnFWTUYyalVHU1VLakhjUUZINFRlOTA?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Employers Seek New Strategies to Rein In Opacity in PBM Pricing</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Despite growing regulatory and market pressure for PBM transparency, employers continue to struggle with opaque pricing structures that inflate drug costs. The article explores actionable strategies for self-funded employers to demand accountability and better manage escalating pharmacy spend.</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>MedCity News</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Wed, 07 Oct 2026 13:45:52 GMT</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxON0UxQ0U3a3kyOVlDdjhVNVZxeFFqZUNNVjJ3cGQ1ckpNeHhMOU5kdnVlbUZQZUNTNXlMblFBMFlrSGN3Ul8xdmhZTFdTSnpiVVNqUGdSYnpUZTB1bHdiZ0c0cDhHWHBWRUVQT0g3QWRCRU1GclB0N0djX3kxUEJSblpZWmJBc0Q5bWIyVTlfaXYzUWRNR3RpVFNzSWxydmVjZllPV1lXN3ZIdw?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Congress Scrutinizes PBM and Broker Payments Amid Employer Drug Market Shifts</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Lawmakers are increasingly focusing on financial arrangements between pharmacy benefit managers and brokers, mirroring broader legislative pushes for transparency in employer-sponsored health plans. This scrutiny directly impacts how self-funded employers evaluate their PBM partnerships and fee structures. As regulatory pressure mounts, plan sponsors will need greater clarity on broker compensation and PBM revenue streams to ensure fiduciary compliance.</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Insurance Business</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Wed, 07 Oct 2026 11:07:25 GMT</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQbkZtNkh0U19Sb3J0MXBVV29qZ0xvbERVMS1OMzMzLW94eFR2UDVqYW16OGxEMlNkSGY3Nzh0bHdaRlhVVEpCM2NuNDFBX1JBeHdUX1VWYVRMamtLU0xuWXlITV9mbGd6bWdqX2V0OUstNlFiMndfaVJ6MWlra3VzdnhrSjRNR3ExUFY3NFhya2FPY3JIRWpCZXdEY1pFeXVWd3hwTWRkZjNhcFhDWElDeUdVUzhxZEJBLWpWelJxOF9RdndEZmpIVlc5Ylo?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Employers Push for PBM Reform and Transparency</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Self-funded employers are increasingly pushing back against traditional pharmacy benefit managers to demand greater pricing transparency and reform. This shift highlights growing employer dissatisfaction with current PBM practices and creates opportunities for alternative, transparent benefit models.</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Human Resources Director</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Wed, 07 Oct 2026 18:30:03 GMT</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxOR3NGUkJFZFdyUHA3ejNDcWVSQWhLSEJCNnptQVhrUVVRUXNHYnBGM1NpeXZ4MmxsZmdCV3pjOXdJVUc4ZlU4S2FEWl9VcG5kdy0wUWRlbWhrWnB3Sk1HQzhlVUpVZWpfNlJCdTFJbTM1OUgxd2xVbjBLZjNjQW5nZnNWbTRILVd6c0RmQW95WGJrVlJEQm9zd3oxWFJZSHd0bTI3Nnk2T2ZjcjZFcndOQi1TY1dXY19OLTZTRUd1NHVZQQ?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Prime Therapeutics Launches New Sales Model Focusing on Upfront Drug Prices</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Prime Therapeutics is introducing a new pharmaceutical sales model that emphasizes upfront drug pricing rather than traditional back-end rebates. This shift directly impacts self-funded employer health plans by changing how net drug costs are calculated and managed. The model represents a broader industry trend toward pricing transparency and alternative PBM compensation structures.</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Bloomberg.com</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Wed, 07 Oct 2026 20:13:14 GMT</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOZkZseGc2bk1sNzFEcnNxVzFhQmdTeVBmc0tmNTlIbm9XSHBIaUdtX3o0dE1DZlI1ZWxfMmRlY28zbS1UMUJURHkzRGZsbzF4MnpXVjJTVjRuR0lLN05VcWJVQl9HMHN3Q0ZSa1lqZkZqRzdfTV9SQXdnc3RrRmlPZW1BMVNEOEU0eXVLd213TkFpNDRqUTktLTFxRElFNXJWdDlmU0JvT2daeVhjSlY3bUNYYktHUQ?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Florida Targets PBM Rebate Aggregators in Insulin Pricing Lawsuit</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>The state of Florida has filed a lawsuit against group purchasing organizations (GPOs) and rebate aggregators that operate behind major pharmacy benefit managers. This legal action targets the complex rebate and fee structures tied to insulin pricing, holding significant implications for PBM transparency, spread pricing, and self-funded employer health plans.</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Business Model Analyst</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Wed, 07 Oct 2026 19:26:51 GMT</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPQVdtelJqeGtRZmRCYUFMV0tPQ0hPYzNTUXI5QUJwSkwxNEtZUlVEdmVPX2d3UmRqNVdWNjY1VVktbHhndmV1OC10MEd4dm1FamFCVFdZUWgwSE9OU3RpMzdmV2phUy1lM0lEa1ZtY2QzeGNDc1lEVW1PSk5lc1N5QTdDWjVOaWc?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Virta Health Hits Profitability Amid Rising Employer Demand for Diabetes Reversal</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Virta Health has achieved profitability and expanded its client base to over 750 organizations, driven by employer demand for chronic condition management solutions. As self-funded employers grapple with escalating pharmacy costs—particularly for diabetes and GLP-1 drugs—point solutions focused on metabolic health and reversal are gaining significant market traction. This growth highlights how employers are increasingly integrating specialized digital health interventions into their benefit plans to manage long-term medical and pharmacy spend.</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Lelezard</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Wed, 07 Oct 2026 04:36:32 GMT</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOOGVYem9ZdU1vdmhBNlRkTUZvU2NPQWFhblgzWG5VbHdDNXBVcUtvQWVVZldqY2Zjb2IzeWFRS1hvT0h2TjVvZU5IMGQtNHJzUDJmM3R3S2NIeEJEV0RybFV4OGwzZGdjdnJpc0pxNkNKU0lUb1ctUC02ZWVUcU1samFDWVJkZ25rSUM3Wk9WM0FuQXlwcmRibkJnWFR6aHFzMzZpRWFsck93S1pNVkc4ZERuRUhVYW41d1BQdVJn?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>McKesson and PE Firm Acquire Option Care Health for Home Infusion Expansion</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>McKesson and a private equity firm have acquired major home infusion provider Option Care Health, signaling a strategic consolidation in the specialty and alternative-site distribution market. For self-funded employers and PBMs, this shift could impact the site-of-care delivery economics and cost management strategies for complex, high-cost specialty therapies.</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Managed Healthcare Executive</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Wed, 07 Oct 2026 09:45:37 GMT</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPdnpYVDBHSENRSTVLVjRRa19UX1FYZE5yYXhBYUttaGhVRHg1QTQwXy14ZERTeXNyRnpybzVSRjVKVjlXTEw4Z01GdFNaT2lxOXE4Wl9DcDR0aGtOU3B5bGROZ2puaUFELWVPY1ZzbmhLemJRbXRTb1VBc3RWSUlXZTF3ZEpwd0I5VWt2RllGSG00djBoVy1sSzhEWVV1Y01LVnh6UUhTOEFBbjFRcFFHXzE2QW1Qc3N6S1R4VlFR?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Prime Therapeutics Launches Upfront Pricing Model for Drug Sales</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Prime Therapeutics is introducing a new drug sales model focused on upfront pricing, shifting away from traditional rebate-heavy structures. This evolution in PBM pricing models directly impacts self-funded employers seeking greater transparency and predictability in their pharmacy benefit costs.</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Modern Healthcare</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Wed, 07 Oct 2026 22:09:00 GMT</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQbGlmTTFJcWlqSDdrU0o1ajBBRzRWUjY3SDZDMDBtZ01fT2MzTWNzWVdLOWxVa3dGXzNjTVhSZHkwYVlDY29pSXhQQl9PM1BoZjIwN0dSdW1VUW1BSzYxclBRaVNPcWxvTXFZYzFfUjdkOTllQXAzVk5YMHpTOVdmcmE0OURqejJ1Z1Rhb1BxSUx5Y2dkODlma1FLRERLZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQX2NmMUROQWZZYXMwakZiXzVDUk5NNnE2TWRFYjJVbkZvc0RBSUNIQUlMQ01GTG5wd1F4WW9qeUdFeW91QkxPOXAxTDVZSEl6Q1ZsTnFhUUhiQmNiTGZwZm9iczUyVnltTnljWmlhUVk2X1RkaHprWXdrUkhMQ3Z1VTc5ZnprZWlYdmlON1FmSWdEb1lUdEdpWXJjTVhpODVtODVzYUtrSnpuZW1Fb3d4VzNtYmpzZw?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>